<commit_message>
Translators 0.4.1 for the Craft releases of 2026-10-13
The canary (issue #2) found that WordCraft 0.6.1, GridCraft 0.6.1, CADCraft 0.6.2 and
EffectCraft 0.9.2 broke saving back, and that the pointer tests of six apps no longer matched.
The adapters, specs and app pages follow the new releases, which become the tested versions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/e2e/fixtures/gridcraft/sales-sample.xlsx
+++ b/tests/e2e/fixtures/gridcraft/sales-sample.xlsx
@@ -1209,7 +1209,11 @@
   </sheetData>
   <conditionalFormatting sqref="H5:H10">
     <cfRule type="iconSet" priority="1">
-      <iconSet iconSet="3Arrows"/>
+      <iconSet iconSet="3Arrows">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G10">

</xml_diff>